<commit_message>
tcc back to 500m according to manuscript methods
</commit_message>
<xml_diff>
--- a/tables/model_outputs.xlsx
+++ b/tables/model_outputs.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="218">
   <si>
     <t xml:space="preserve">part</t>
   </si>
@@ -92,16 +92,16 @@
     <t xml:space="preserve"/>
   </si>
   <si>
-    <t xml:space="preserve">0.293</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-5.230</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-1.000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.072</t>
+    <t xml:space="preserve">0.265</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-5.045</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.251</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.078</t>
   </si>
   <si>
     <t xml:space="preserve">conf.int</t>
@@ -128,16 +128,16 @@
     <t xml:space="preserve">[0.751, 1.110]</t>
   </si>
   <si>
-    <t xml:space="preserve">[-0.564, 1.005]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[-13.868, 4.799]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[-5.300, 3.243]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[-0.226, 0.091]</t>
+    <t xml:space="preserve">[-0.777, 1.150]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[-18.857, 8.079]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[-16.620, 17.425]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[-0.233, 0.072]</t>
   </si>
   <si>
     <t xml:space="preserve">b_imp200m_s</t>
@@ -332,16 +332,16 @@
     <t xml:space="preserve">0.367</t>
   </si>
   <si>
-    <t xml:space="preserve">1.604</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10.694</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.594</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.353</t>
+    <t xml:space="preserve">1.840</t>
+  </si>
+  <si>
+    <t xml:space="preserve">28.023</t>
+  </si>
+  <si>
+    <t xml:space="preserve">33.323</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.342</t>
   </si>
   <si>
     <t xml:space="preserve">[0.318, 0.499]</t>
@@ -350,304 +350,298 @@
     <t xml:space="preserve">[0.295, 0.465]</t>
   </si>
   <si>
-    <t xml:space="preserve">[0.848, 2.624]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[6.074, 17.779]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[3.137, 9.518]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[0.258, 0.529]</t>
+    <t xml:space="preserve">[0.949, 3.062]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[18.198, 42.526]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[13.072, 54.305]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[0.253, 0.506]</t>
   </si>
   <si>
     <t xml:space="preserve">b_beeshannons_Intercept</t>
   </si>
   <si>
-    <t xml:space="preserve">0.229</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[-0.250, 0.677]</t>
+    <t xml:space="preserve">-0.000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[-0.349, 0.337]</t>
   </si>
   <si>
     <t xml:space="preserve">b_beeshannons_imp200m_s</t>
   </si>
   <si>
-    <t xml:space="preserve">-0.580</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[-0.914, -0.206]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">b_beeshannons_WealthIndex_s</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.054</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[-0.454, 0.352]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">b_beeshannons_IWealthIndex_sE2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.226</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[-0.536, 0.082]</t>
+    <t xml:space="preserve">-0.526</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[-0.890, -0.150]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bs_beeshannons_sWealthIndex_s_1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.195</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[-0.930, 0.602]</t>
   </si>
   <si>
     <t xml:space="preserve">sigma_beeshannons</t>
   </si>
   <si>
-    <t xml:space="preserve">0.808</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[0.599, 1.145]</t>
+    <t xml:space="preserve">0.822</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[0.613, 1.173]</t>
   </si>
   <si>
     <t xml:space="preserve">b_deltano_Intercept</t>
   </si>
   <si>
+    <t xml:space="preserve">0.276</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[-0.720, 1.123]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b_deltano_bee.shannon_s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.190</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[0.265, 2.090]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sigma_deltano</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.821</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[1.066, 2.907]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b_bee.shannon_s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.210</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.812</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-4.901</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.095</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[0.204, 2.235]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[-9.912, 12.970]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[-20.957, 11.134]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[-0.244, 0.056]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b_n.pol_s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.572</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-9.675</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.323</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.080</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[-1.542, 0.474]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[-21.480, 3.781]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[-13.548, 20.792]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[-0.236, 0.083]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b_n.herb_s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.460</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.483</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.023</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.124</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[-0.752, 1.723]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[-9.531, 16.727]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[-12.874, 26.505]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[-0.059, 0.303]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b_n.enemy_s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.821</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-6.849</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.012</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[-1.249, 1.108]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[-13.318, 11.519]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[-27.778, 9.915]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[-0.182, 0.162]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sd_site_code__Intercept</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.333</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.312</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.542</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.171</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.094</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.150</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.174</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[0.190, 0.537]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[0.027, 0.615]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[0.097, 0.931]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[0.008, 0.410]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[0.004, 0.287]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[0.008, 0.329]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[0.016, 0.353]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gof</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Num.Obs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">63</t>
+  </si>
+  <si>
+    <t xml:space="preserve">59</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.678</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.523</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.443</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.440</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.525</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.466</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.415</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.288</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.161</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.131</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.247</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R2 Marg.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.493</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.416</t>
+  </si>
+  <si>
     <t xml:space="preserve">0.254</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[-0.711, 1.055]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">b_deltano_bee.shannon_s</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.173</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[0.283, 2.011]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sigma_deltano</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.681</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[0.976, 2.648]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">b_bee.shannon_s</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.039</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.112</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.262</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.107</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[0.177, 1.866]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[-1.885, 2.078]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[-2.078, 1.561]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[-0.267, 0.063]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">b_n.pol_s</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.474</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.473</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.381</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.096</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[-1.229, 0.386]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[-2.398, 1.512]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[-1.337, 2.101]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[-0.283, 0.088]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">b_n.herb_s</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.366</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.055</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.391</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.162</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[-0.627, 1.326]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[-2.027, 1.906]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[-1.427, 2.199]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[-0.068, 0.387]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">b_n.enemy_s</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.101</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.078</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.098</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.032</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[-0.827, 0.961]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[-2.097, 1.910]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[-1.916, 1.708]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[-0.227, 0.180]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sd_site_code__Intercept</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.333</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.312</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.542</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.171</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.094</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.150</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.174</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[0.190, 0.537]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[0.027, 0.615]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[0.097, 0.931]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[0.008, 0.410]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[0.004, 0.287]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[0.008, 0.329]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[0.016, 0.353]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gof</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Num.Obs.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">63</t>
-  </si>
-  <si>
-    <t xml:space="preserve">59</t>
-  </si>
-  <si>
-    <t xml:space="preserve">21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.678</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.523</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.443</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.440</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.525</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.466</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.415</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.233</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.301</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R2 Marg.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.493</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.416</t>
   </si>
   <si>
     <t xml:space="preserve">0.385</t>
@@ -2395,19 +2389,19 @@
         <v>25</v>
       </c>
       <c r="K30" t="s">
+        <v>25</v>
+      </c>
+      <c r="L30" t="s">
         <v>138</v>
       </c>
-      <c r="L30" t="s">
-        <v>25</v>
-      </c>
       <c r="M30" t="s">
-        <v>25</v>
+        <v>139</v>
       </c>
       <c r="N30" t="s">
-        <v>25</v>
+        <v>140</v>
       </c>
       <c r="O30" t="s">
-        <v>25</v>
+        <v>141</v>
       </c>
     </row>
     <row r="31">
@@ -2442,19 +2436,19 @@
         <v>25</v>
       </c>
       <c r="K31" t="s">
-        <v>139</v>
+        <v>25</v>
       </c>
       <c r="L31" t="s">
-        <v>25</v>
+        <v>142</v>
       </c>
       <c r="M31" t="s">
-        <v>25</v>
+        <v>143</v>
       </c>
       <c r="N31" t="s">
-        <v>25</v>
+        <v>144</v>
       </c>
       <c r="O31" t="s">
-        <v>25</v>
+        <v>145</v>
       </c>
     </row>
     <row r="32">
@@ -2462,7 +2456,7 @@
         <v>15</v>
       </c>
       <c r="B32" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="C32" t="s">
         <v>17</v>
@@ -2492,16 +2486,16 @@
         <v>25</v>
       </c>
       <c r="L32" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="M32" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="N32" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="O32" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
     </row>
     <row r="33">
@@ -2509,7 +2503,7 @@
         <v>15</v>
       </c>
       <c r="B33" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="C33" t="s">
         <v>30</v>
@@ -2539,16 +2533,16 @@
         <v>25</v>
       </c>
       <c r="L33" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="M33" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="N33" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="O33" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
     </row>
     <row r="34">
@@ -2556,7 +2550,7 @@
         <v>15</v>
       </c>
       <c r="B34" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="C34" t="s">
         <v>17</v>
@@ -2586,16 +2580,16 @@
         <v>25</v>
       </c>
       <c r="L34" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="M34" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="N34" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="O34" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
     </row>
     <row r="35">
@@ -2603,7 +2597,7 @@
         <v>15</v>
       </c>
       <c r="B35" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="C35" t="s">
         <v>30</v>
@@ -2633,16 +2627,16 @@
         <v>25</v>
       </c>
       <c r="L35" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="M35" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="N35" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="O35" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
     </row>
     <row r="36">
@@ -2650,7 +2644,7 @@
         <v>15</v>
       </c>
       <c r="B36" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="C36" t="s">
         <v>17</v>
@@ -2680,16 +2674,16 @@
         <v>25</v>
       </c>
       <c r="L36" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="M36" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="N36" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="O36" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
     </row>
     <row r="37">
@@ -2697,7 +2691,7 @@
         <v>15</v>
       </c>
       <c r="B37" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="C37" t="s">
         <v>30</v>
@@ -2727,16 +2721,16 @@
         <v>25</v>
       </c>
       <c r="L37" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="M37" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="N37" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="O37" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
     </row>
     <row r="38">
@@ -2744,46 +2738,46 @@
         <v>15</v>
       </c>
       <c r="B38" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="C38" t="s">
         <v>17</v>
       </c>
       <c r="D38" t="s">
-        <v>25</v>
+        <v>174</v>
       </c>
       <c r="E38" t="s">
-        <v>25</v>
+        <v>175</v>
       </c>
       <c r="F38" t="s">
-        <v>25</v>
+        <v>176</v>
       </c>
       <c r="G38" t="s">
-        <v>25</v>
+        <v>177</v>
       </c>
       <c r="H38" t="s">
-        <v>25</v>
+        <v>178</v>
       </c>
       <c r="I38" t="s">
-        <v>25</v>
+        <v>179</v>
       </c>
       <c r="J38" t="s">
-        <v>25</v>
+        <v>180</v>
       </c>
       <c r="K38" t="s">
         <v>25</v>
       </c>
       <c r="L38" t="s">
-        <v>168</v>
+        <v>25</v>
       </c>
       <c r="M38" t="s">
-        <v>169</v>
+        <v>25</v>
       </c>
       <c r="N38" t="s">
-        <v>170</v>
+        <v>25</v>
       </c>
       <c r="O38" t="s">
-        <v>171</v>
+        <v>25</v>
       </c>
     </row>
     <row r="39">
@@ -2791,269 +2785,269 @@
         <v>15</v>
       </c>
       <c r="B39" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="C39" t="s">
         <v>30</v>
       </c>
       <c r="D39" t="s">
-        <v>25</v>
+        <v>181</v>
       </c>
       <c r="E39" t="s">
-        <v>25</v>
+        <v>182</v>
       </c>
       <c r="F39" t="s">
-        <v>25</v>
+        <v>183</v>
       </c>
       <c r="G39" t="s">
-        <v>25</v>
+        <v>184</v>
       </c>
       <c r="H39" t="s">
-        <v>25</v>
+        <v>185</v>
       </c>
       <c r="I39" t="s">
-        <v>25</v>
+        <v>186</v>
       </c>
       <c r="J39" t="s">
-        <v>25</v>
+        <v>187</v>
       </c>
       <c r="K39" t="s">
         <v>25</v>
       </c>
       <c r="L39" t="s">
-        <v>172</v>
+        <v>25</v>
       </c>
       <c r="M39" t="s">
-        <v>173</v>
+        <v>25</v>
       </c>
       <c r="N39" t="s">
-        <v>174</v>
+        <v>25</v>
       </c>
       <c r="O39" t="s">
-        <v>175</v>
+        <v>25</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>15</v>
+        <v>188</v>
       </c>
       <c r="B40" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="C40" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="D40" t="s">
-        <v>177</v>
+        <v>190</v>
       </c>
       <c r="E40" t="s">
-        <v>178</v>
+        <v>190</v>
       </c>
       <c r="F40" t="s">
-        <v>179</v>
+        <v>190</v>
       </c>
       <c r="G40" t="s">
-        <v>180</v>
+        <v>190</v>
       </c>
       <c r="H40" t="s">
-        <v>181</v>
+        <v>191</v>
       </c>
       <c r="I40" t="s">
-        <v>182</v>
+        <v>191</v>
       </c>
       <c r="J40" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="K40" t="s">
-        <v>25</v>
+        <v>192</v>
       </c>
       <c r="L40" t="s">
-        <v>25</v>
+        <v>192</v>
       </c>
       <c r="M40" t="s">
-        <v>25</v>
+        <v>193</v>
       </c>
       <c r="N40" t="s">
-        <v>25</v>
+        <v>193</v>
       </c>
       <c r="O40" t="s">
-        <v>25</v>
+        <v>193</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>15</v>
+        <v>188</v>
       </c>
       <c r="B41" t="s">
-        <v>176</v>
+        <v>194</v>
       </c>
       <c r="C41" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="D41" t="s">
-        <v>184</v>
+        <v>195</v>
       </c>
       <c r="E41" t="s">
-        <v>185</v>
+        <v>196</v>
       </c>
       <c r="F41" t="s">
-        <v>186</v>
+        <v>197</v>
       </c>
       <c r="G41" t="s">
-        <v>187</v>
+        <v>198</v>
       </c>
       <c r="H41" t="s">
-        <v>188</v>
+        <v>199</v>
       </c>
       <c r="I41" t="s">
-        <v>189</v>
+        <v>200</v>
       </c>
       <c r="J41" t="s">
-        <v>190</v>
+        <v>201</v>
       </c>
       <c r="K41" t="s">
         <v>25</v>
       </c>
       <c r="L41" t="s">
-        <v>25</v>
+        <v>202</v>
       </c>
       <c r="M41" t="s">
-        <v>25</v>
+        <v>203</v>
       </c>
       <c r="N41" t="s">
-        <v>25</v>
+        <v>204</v>
       </c>
       <c r="O41" t="s">
-        <v>25</v>
+        <v>205</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="B42" t="s">
-        <v>192</v>
+        <v>206</v>
       </c>
       <c r="C42" t="s">
         <v>25</v>
       </c>
       <c r="D42" t="s">
-        <v>193</v>
+        <v>207</v>
       </c>
       <c r="E42" t="s">
-        <v>193</v>
+        <v>208</v>
       </c>
       <c r="F42" t="s">
-        <v>193</v>
+        <v>209</v>
       </c>
       <c r="G42" t="s">
-        <v>193</v>
+        <v>210</v>
       </c>
       <c r="H42" t="s">
-        <v>194</v>
+        <v>211</v>
       </c>
       <c r="I42" t="s">
-        <v>194</v>
+        <v>212</v>
       </c>
       <c r="J42" t="s">
-        <v>194</v>
+        <v>213</v>
       </c>
       <c r="K42" t="s">
-        <v>195</v>
+        <v>25</v>
       </c>
       <c r="L42" t="s">
-        <v>195</v>
+        <v>25</v>
       </c>
       <c r="M42" t="s">
-        <v>196</v>
+        <v>25</v>
       </c>
       <c r="N42" t="s">
-        <v>196</v>
+        <v>25</v>
       </c>
       <c r="O42" t="s">
-        <v>196</v>
+        <v>25</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="B43" t="s">
-        <v>197</v>
+        <v>214</v>
       </c>
       <c r="C43" t="s">
         <v>25</v>
       </c>
       <c r="D43" t="s">
-        <v>198</v>
+        <v>25</v>
       </c>
       <c r="E43" t="s">
-        <v>199</v>
+        <v>25</v>
       </c>
       <c r="F43" t="s">
-        <v>200</v>
+        <v>25</v>
       </c>
       <c r="G43" t="s">
-        <v>201</v>
+        <v>25</v>
       </c>
       <c r="H43" t="s">
-        <v>202</v>
+        <v>25</v>
       </c>
       <c r="I43" t="s">
-        <v>203</v>
+        <v>25</v>
       </c>
       <c r="J43" t="s">
-        <v>204</v>
+        <v>25</v>
       </c>
       <c r="K43" t="s">
-        <v>25</v>
+        <v>215</v>
       </c>
       <c r="L43" t="s">
-        <v>205</v>
+        <v>25</v>
       </c>
       <c r="M43" t="s">
-        <v>206</v>
+        <v>25</v>
       </c>
       <c r="N43" t="s">
-        <v>207</v>
+        <v>25</v>
       </c>
       <c r="O43" t="s">
-        <v>208</v>
+        <v>25</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="B44" t="s">
-        <v>209</v>
+        <v>216</v>
       </c>
       <c r="C44" t="s">
         <v>25</v>
       </c>
       <c r="D44" t="s">
-        <v>210</v>
+        <v>25</v>
       </c>
       <c r="E44" t="s">
-        <v>211</v>
+        <v>25</v>
       </c>
       <c r="F44" t="s">
-        <v>132</v>
+        <v>25</v>
       </c>
       <c r="G44" t="s">
-        <v>212</v>
+        <v>25</v>
       </c>
       <c r="H44" t="s">
-        <v>213</v>
+        <v>25</v>
       </c>
       <c r="I44" t="s">
-        <v>214</v>
+        <v>25</v>
       </c>
       <c r="J44" t="s">
-        <v>215</v>
+        <v>25</v>
       </c>
       <c r="K44" t="s">
-        <v>25</v>
+        <v>217</v>
       </c>
       <c r="L44" t="s">
         <v>25</v>
@@ -3065,100 +3059,6 @@
         <v>25</v>
       </c>
       <c r="O44" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="s">
-        <v>191</v>
-      </c>
-      <c r="B45" t="s">
-        <v>216</v>
-      </c>
-      <c r="C45" t="s">
-        <v>25</v>
-      </c>
-      <c r="D45" t="s">
-        <v>25</v>
-      </c>
-      <c r="E45" t="s">
-        <v>25</v>
-      </c>
-      <c r="F45" t="s">
-        <v>25</v>
-      </c>
-      <c r="G45" t="s">
-        <v>25</v>
-      </c>
-      <c r="H45" t="s">
-        <v>25</v>
-      </c>
-      <c r="I45" t="s">
-        <v>25</v>
-      </c>
-      <c r="J45" t="s">
-        <v>25</v>
-      </c>
-      <c r="K45" t="s">
-        <v>217</v>
-      </c>
-      <c r="L45" t="s">
-        <v>25</v>
-      </c>
-      <c r="M45" t="s">
-        <v>25</v>
-      </c>
-      <c r="N45" t="s">
-        <v>25</v>
-      </c>
-      <c r="O45" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="s">
-        <v>191</v>
-      </c>
-      <c r="B46" t="s">
-        <v>218</v>
-      </c>
-      <c r="C46" t="s">
-        <v>25</v>
-      </c>
-      <c r="D46" t="s">
-        <v>25</v>
-      </c>
-      <c r="E46" t="s">
-        <v>25</v>
-      </c>
-      <c r="F46" t="s">
-        <v>25</v>
-      </c>
-      <c r="G46" t="s">
-        <v>25</v>
-      </c>
-      <c r="H46" t="s">
-        <v>25</v>
-      </c>
-      <c r="I46" t="s">
-        <v>25</v>
-      </c>
-      <c r="J46" t="s">
-        <v>25</v>
-      </c>
-      <c r="K46" t="s">
-        <v>219</v>
-      </c>
-      <c r="L46" t="s">
-        <v>25</v>
-      </c>
-      <c r="M46" t="s">
-        <v>25</v>
-      </c>
-      <c r="N46" t="s">
-        <v>25</v>
-      </c>
-      <c r="O46" t="s">
         <v>25</v>
       </c>
     </row>

</xml_diff>